<commit_message>
data: hourly update 2026-07-09 19:59Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-07-09.xlsx
+++ b/data/output/workbook/2026-07-09.xlsx
@@ -401,7 +401,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="10925175"/>
+    <ext cx="10125075" cy="10753725"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09 14:59</t>
+          <t>2026-07-09 15:58</t>
         </is>
       </c>
     </row>
@@ -8836,10 +8836,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.6347</v>
+        <v>0.6375999999999999</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-174</v>
+        <v>-176</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>170</v>
@@ -8866,7 +8866,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 63.8% (fair -176). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8949,32 +8949,32 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies @ Cincinnati Reds</t>
+          <t>Boston Red Sox @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.7412000000000001</v>
+        <v>0.5644</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-286</v>
+        <v>-130</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-153</v>
+        <v>120</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 74.1% (fair -286). Your call.</t>
+          <t>Model 56.4% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -9015,32 +9015,32 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Athletics @ Detroit Tigers</t>
+          <t>Seattle Storm @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Seattle Storm</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5361</v>
+        <v>0.2065</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-116</v>
+        <v>384</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>127</v>
+        <v>495</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -116). Your call.</t>
+          <t>Model 20.7% (fair +384). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -9081,32 +9081,32 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Boston Red Sox @ Chicago White Sox</t>
+          <t>Philadelphia Phillies @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5528</v>
+        <v>0.7412000000000001</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-124</v>
+        <v>-286</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>120</v>
+        <v>-153</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9130,7 +9130,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 74.1% (fair -286). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -9166,10 +9166,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.582</v>
+        <v>0.5770999999999999</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-139</v>
+        <v>-136</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>104</v>
@@ -9196,7 +9196,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -9213,12 +9213,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Atlanta Dream</t>
+          <t>Indiana Fever @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -9228,17 +9228,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.2114</v>
+        <v>0.5663</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>373</v>
+        <v>-131</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>456</v>
+        <v>104</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9262,7 +9262,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 21.1% (fair +373). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9274,37 +9274,37 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Indiana Fever @ Phoenix Mercury</t>
+          <t>Golden State Valkyries @ Connecticut Sun</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Over 154.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5639000000000001</v>
+        <v>0.5767</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-129</v>
+        <v>-136</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -129). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9345,12 +9345,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Golden State Valkyries @ Connecticut Sun</t>
+          <t>Atlanta Braves @ St. Louis Cardinals</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>00:15</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -9360,17 +9360,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 154.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5816</v>
+        <v>0.5575</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-139</v>
+        <v>-126</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-104</v>
+        <v>105</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9394,7 +9394,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 55.8% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9406,37 +9406,37 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees @ Washington Nationals</t>
+          <t>Seattle Mariners @ Miami Marlins</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4796</v>
+        <v>0.5288</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>109</v>
+        <v>-112</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +109). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -9472,37 +9472,37 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Miami Marlins</t>
+          <t>New York Yankees @ Washington Nationals</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5288</v>
+        <v>0.4771</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-112</v>
+        <v>110</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 47.7% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -9543,32 +9543,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings @ Toronto Tempo</t>
+          <t>Kansas City Royals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo +6.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5415</v>
+        <v>0.5616</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-118</v>
+        <v>-128</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -9592,7 +9592,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -9628,7 +9628,7 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5598000000000001</v>
+        <v>0.5604</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>-127</v>
@@ -9675,12 +9675,12 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ New York Mets</t>
+          <t>Las Vegas Aces @ Portland Fire</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -9690,17 +9690,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5434</v>
+        <v>0.5476</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-119</v>
+        <v>-121</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9724,7 +9724,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9736,17 +9736,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Braves @ St. Louis Cardinals</t>
+          <t>Kansas City Royals @ New York Mets</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>00:15</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9756,17 +9756,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5575</v>
+        <v>0.542</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-126</v>
+        <v>-118</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9790,7 +9790,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 55.8% (fair -126). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9802,37 +9802,37 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Los Angeles Sparks</t>
+          <t>Athletics @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5541</v>
+        <v>0.5182</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-124</v>
+        <v>-108</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-104</v>
+        <v>113</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9856,7 +9856,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 55.4% (fair -124). Your call.</t>
+          <t>Model 51.8% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9873,12 +9873,12 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Houston Astros @ Texas Rangers</t>
+          <t>Dallas Wings @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -9888,17 +9888,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Toronto Tempo</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4894</v>
+        <v>0.2999</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>104</v>
+        <v>233</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>122</v>
+        <v>264</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9922,7 +9922,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +104). Your call.</t>
+          <t>Model 30.0% (fair +233). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9939,32 +9939,32 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky @ Los Angeles Sparks</t>
+          <t>Houston Astros @ Texas Rangers</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 180.5</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5422</v>
+        <v>0.4894</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-118</v>
+        <v>104</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9988,7 +9988,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 48.9% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -10005,12 +10005,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings @ Toronto Tempo</t>
+          <t>Chicago Sky @ Los Angeles Sparks</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -10020,17 +10020,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Los Angeles Sparks</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.3018</v>
+        <v>0.5528999999999999</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>231</v>
+        <v>-124</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>257</v>
+        <v>-104</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 30.2% (fair +231). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10071,32 +10071,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Cincinnati Reds</t>
+          <t>Dallas Wings @ Toronto Tempo</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Toronto Tempo +6.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5057</v>
+        <v>0.5522</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-102</v>
+        <v>-123</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>113</v>
+        <v>-104</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10120,7 +10120,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -102). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10203,32 +10203,32 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Atlanta Dream</t>
+          <t>Milwaukee Brewers @ St. Louis Cardinals</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>23:45</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Over 168.5</t>
+          <t>St. Louis Cardinals</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.537</v>
+        <v>0.4764</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-116</v>
+        <v>110</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10264,37 +10264,37 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers @ St. Louis Cardinals</t>
+          <t>Chicago Cubs @ Cincinnati Reds</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:45</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4754</v>
+        <v>0.5151</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>110</v>
+        <v>-106</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -10318,7 +10318,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -10335,32 +10335,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies @ Cincinnati Reds</t>
+          <t>Athletics @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies -1.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5286</v>
+        <v>0.4818</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-112</v>
+        <v>108</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -10384,7 +10384,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 48.2% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -10396,17 +10396,17 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Cincinnati Reds</t>
+          <t>Seattle Storm @ Atlanta Dream</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -10416,17 +10416,17 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 168.5</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5119</v>
+        <v>0.5395</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-105</v>
+        <v>-117</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>108</v>
+        <v>-102</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -11023,7 +11023,7 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4353</v>
+        <v>0.4343</v>
       </c>
       <c r="G11" s="14" t="n">
         <v>130</v>
@@ -11053,7 +11053,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 43.5% (fair +130). Your call.</t>
+          <t>Model 43.4% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -11089,7 +11089,7 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5647</v>
+        <v>0.5657</v>
       </c>
       <c r="G12" s="14" t="n">
         <v>-130</v>
@@ -11119,7 +11119,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 56.5% (fair -130). Your call.</t>
+          <t>Model 56.6% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -11155,10 +11155,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4566</v>
+        <v>0.458</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>113</v>
@@ -11185,7 +11185,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 45.7% (fair +119). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -11221,10 +11221,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5434</v>
+        <v>0.542</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-119</v>
+        <v>-118</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>106</v>
@@ -11251,7 +11251,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 54.3% (fair -119). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -11287,10 +11287,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.3908</v>
+        <v>0.3921</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>153</v>
@@ -11317,7 +11317,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 39.1% (fair +156). Your call.</t>
+          <t>Model 39.2% (fair +155). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -11353,10 +11353,10 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.6092</v>
+        <v>0.6079</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-156</v>
+        <v>-155</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>-156</v>
@@ -11383,7 +11383,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 60.9% (fair -156). Your call.</t>
+          <t>Model 60.8% (fair -155). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -11815,7 +11815,7 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4576</v>
+        <v>0.4566</v>
       </c>
       <c r="G23" s="14" t="n">
         <v>119</v>
@@ -11845,7 +11845,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +119). Your call.</t>
+          <t>Model 45.7% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -11881,7 +11881,7 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5424</v>
+        <v>0.5434</v>
       </c>
       <c r="G24" s="14" t="n">
         <v>-119</v>
@@ -11911,7 +11911,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -119). Your call.</t>
+          <t>Model 54.3% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11947,10 +11947,10 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4522</v>
+        <v>0.4512</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H25" s="15" t="n">
         <v>102</v>
@@ -11977,7 +11977,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -12013,10 +12013,10 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4658</v>
+        <v>0.4667999999999999</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>106</v>
@@ -12043,7 +12043,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 46.7% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -12079,7 +12079,7 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.3652</v>
+        <v>0.3653</v>
       </c>
       <c r="G27" s="14" t="n">
         <v>174</v>
@@ -12145,7 +12145,7 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.6348</v>
+        <v>0.6347</v>
       </c>
       <c r="G28" s="14" t="n">
         <v>-174</v>
@@ -12607,7 +12607,7 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4831</v>
+        <v>0.4832</v>
       </c>
       <c r="G35" s="14" t="n">
         <v>107</v>
@@ -12673,7 +12673,7 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5169</v>
+        <v>0.5168</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>-107</v>
@@ -12739,10 +12739,10 @@
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.4472</v>
+        <v>0.4356</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="H37" s="15" t="n">
         <v>117</v>
@@ -12769,7 +12769,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 43.6% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -12805,10 +12805,10 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.5528</v>
+        <v>0.5644</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-124</v>
+        <v>-130</v>
       </c>
       <c r="H38" s="15" t="n">
         <v>120</v>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 56.4% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -12871,10 +12871,10 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.3653</v>
+        <v>0.3624</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H39" s="15" t="n">
         <v>170</v>
@@ -12901,7 +12901,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 36.5% (fair +174). Your call.</t>
+          <t>Model 36.2% (fair +176). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12937,10 +12937,10 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.6347</v>
+        <v>0.6375999999999999</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>-174</v>
+        <v>-176</v>
       </c>
       <c r="H40" s="15" t="n">
         <v>170</v>
@@ -12967,7 +12967,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 63.8% (fair -176). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -13003,10 +13003,10 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.4477</v>
+        <v>0.4586</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H41" s="15" t="n">
         <v>117</v>
@@ -13033,7 +13033,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 44.8% (fair +123). Your call.</t>
+          <t>Model 45.9% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -13069,10 +13069,10 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5523</v>
+        <v>0.5414</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-123</v>
+        <v>-118</v>
       </c>
       <c r="H42" s="15" t="n">
         <v>-117</v>
@@ -13099,7 +13099,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 54.1% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -13135,13 +13135,13 @@
         </is>
       </c>
       <c r="F43" s="13" t="n">
-        <v>0.5361</v>
+        <v>0.4818</v>
       </c>
       <c r="G43" s="14" t="n">
-        <v>-116</v>
+        <v>108</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -13165,7 +13165,7 @@
       </c>
       <c r="N43" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -116). Your call.</t>
+          <t>Model 48.2% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O43" s="15" t="n"/>
@@ -13201,13 +13201,13 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.4639</v>
+        <v>0.5182</v>
       </c>
       <c r="G44" s="14" t="n">
-        <v>116</v>
+        <v>-108</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="N44" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +116). Your call.</t>
+          <t>Model 51.8% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O44" s="15" t="n"/>
@@ -13267,13 +13267,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.3838</v>
+        <v>0.3682</v>
       </c>
       <c r="G45" s="14" t="n">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -13297,7 +13297,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 38.4% (fair +161). Your call.</t>
+          <t>Model 36.8% (fair +172). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -13333,13 +13333,13 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.6162000000000001</v>
+        <v>0.6317999999999999</v>
       </c>
       <c r="G46" s="14" t="n">
-        <v>-161</v>
+        <v>-172</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-170</v>
+        <v>-163</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -13363,7 +13363,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 61.6% (fair -161). Your call.</t>
+          <t>Model 63.2% (fair -172). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -13399,13 +13399,13 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.5038</v>
+        <v>0.5065999999999999</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>-115</v>
+        <v>-117</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -13429,7 +13429,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -13465,13 +13465,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4962</v>
+        <v>0.4934</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -13495,7 +13495,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -13537,7 +13537,7 @@
         <v>-112</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -13603,7 +13603,7 @@
         <v>112</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -13927,13 +13927,13 @@
         </is>
       </c>
       <c r="F55" s="13" t="n">
-        <v>0.4283</v>
+        <v>0.4159</v>
       </c>
       <c r="G55" s="14" t="n">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -13957,7 +13957,7 @@
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>Model 42.8% (fair +133). Your call.</t>
+          <t>Model 41.6% (fair +140). Your call.</t>
         </is>
       </c>
       <c r="O55" s="15" t="n"/>
@@ -13993,10 +13993,10 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4897</v>
+        <v>0.5025000000000001</v>
       </c>
       <c r="G56" s="14" t="n">
-        <v>104</v>
+        <v>-101</v>
       </c>
       <c r="H56" s="15" t="n">
         <v>-113</v>
@@ -14023,7 +14023,7 @@
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O56" s="15" t="n"/>
@@ -14059,10 +14059,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.4714</v>
+        <v>0.4757</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>-104</v>
@@ -14089,7 +14089,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -14125,10 +14125,10 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.5286</v>
+        <v>0.5243</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="H58" s="15" t="n">
         <v>102</v>
@@ -14155,7 +14155,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 52.4% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -14191,7 +14191,7 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5246</v>
+        <v>0.5236000000000001</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>-110</v>
@@ -14221,7 +14221,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 52.4% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -14257,7 +14257,7 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4754</v>
+        <v>0.4764</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>110</v>
@@ -14287,7 +14287,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -14323,10 +14323,10 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.4901</v>
+        <v>0.4931</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H61" s="15" t="n">
         <v>104</v>
@@ -14353,7 +14353,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -14389,10 +14389,10 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.5099</v>
+        <v>0.5069</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>-104</v>
+        <v>-103</v>
       </c>
       <c r="H62" s="15" t="n">
         <v>-101</v>
@@ -14419,7 +14419,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -14455,7 +14455,7 @@
         </is>
       </c>
       <c r="F63" s="13" t="n">
-        <v>0.5808</v>
+        <v>0.5819</v>
       </c>
       <c r="G63" s="14" t="n">
         <v>-139</v>
@@ -14485,7 +14485,7 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>Model 58.1% (fair -139). Your call.</t>
+          <t>Model 58.2% (fair -139). Your call.</t>
         </is>
       </c>
       <c r="O63" s="15" t="n"/>
@@ -14521,7 +14521,7 @@
         </is>
       </c>
       <c r="F64" s="13" t="n">
-        <v>0.4192</v>
+        <v>0.4181</v>
       </c>
       <c r="G64" s="14" t="n">
         <v>139</v>
@@ -14551,7 +14551,7 @@
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>Model 41.9% (fair +139). Your call.</t>
+          <t>Model 41.8% (fair +139). Your call.</t>
         </is>
       </c>
       <c r="O64" s="15" t="n"/>
@@ -15235,13 +15235,13 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.5204</v>
+        <v>0.5228999999999999</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>-109</v>
+        <v>-110</v>
       </c>
       <c r="H75" s="15" t="n">
-        <v>-133</v>
+        <v>-138</v>
       </c>
       <c r="I75" s="13">
         <f>IF($H$75="","",IF($H$75&lt;0,-$H$75/(-$H$75+100),100/($H$75+100)))</f>
@@ -15265,7 +15265,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -109). Your call.</t>
+          <t>Model 52.3% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -15301,10 +15301,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.4796</v>
+        <v>0.4771</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>136</v>
@@ -15331,7 +15331,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +109). Your call.</t>
+          <t>Model 47.7% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -15763,10 +15763,10 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.4643</v>
+        <v>0.4384</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="H83" s="15" t="n">
         <v>113</v>
@@ -15793,7 +15793,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +115). Your call.</t>
+          <t>Model 43.8% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15829,13 +15829,13 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.5357000000000001</v>
+        <v>0.5616</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-115</v>
+        <v>-128</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I84" s="13">
         <f>IF($H$84="","",IF($H$84&lt;0,-$H$84/(-$H$84+100),100/($H$84+100)))</f>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 56.2% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -16027,10 +16027,10 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.5057</v>
+        <v>0.5567800000000001</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>-102</v>
+        <v>-126</v>
       </c>
       <c r="H87" s="15" t="n">
         <v>113</v>
@@ -16057,7 +16057,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 50.6% (fair -102). Your call.</t>
+          <t>Model 55.7% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -16093,13 +16093,13 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.4943</v>
+        <v>0.44322</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="H88" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I88" s="13">
         <f>IF($H$88="","",IF($H$88&lt;0,-$H$88/(-$H$88+100),100/($H$88+100)))</f>
@@ -16123,7 +16123,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 49.4% (fair +102). Your call.</t>
+          <t>Model 44.3% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -16159,10 +16159,10 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.5119</v>
+        <v>0.5151</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H89" s="15" t="n">
         <v>108</v>
@@ -16189,7 +16189,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -16225,13 +16225,13 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.4881</v>
+        <v>0.4849</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H90" s="15" t="n">
-        <v>-120</v>
+        <v>-115</v>
       </c>
       <c r="I90" s="13">
         <f>IF($H$90="","",IF($H$90&lt;0,-$H$90/(-$H$90+100),100/($H$90+100)))</f>
@@ -16255,7 +16255,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>
@@ -16423,13 +16423,13 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.474</v>
+        <v>0.4802999999999999</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H93" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I93" s="13">
         <f>IF($H$93="","",IF($H$93&lt;0,-$H$93/(-$H$93+100),100/($H$93+100)))</f>
@@ -16453,7 +16453,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -16489,13 +16489,13 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.526</v>
+        <v>0.5197000000000001</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="H94" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I94" s="13">
         <f>IF($H$94="","",IF($H$94&lt;0,-$H$94/(-$H$94+100),100/($H$94+100)))</f>
@@ -16519,7 +16519,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 52.0% (fair -108). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -16555,13 +16555,13 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>0.4875</v>
+        <v>0.4841</v>
       </c>
       <c r="G95" s="14" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H95" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I95" s="13">
         <f>IF($H$95="","",IF($H$95&lt;0,-$H$95/(-$H$95+100),100/($H$95+100)))</f>
@@ -16585,7 +16585,7 @@
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O95" s="15" t="n"/>
@@ -16621,10 +16621,10 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.5125</v>
+        <v>0.5159</v>
       </c>
       <c r="G96" s="14" t="n">
-        <v>-105</v>
+        <v>-107</v>
       </c>
       <c r="H96" s="15" t="n">
         <v>100</v>
@@ -16651,7 +16651,7 @@
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O96" s="15" t="n"/>
@@ -16687,13 +16687,13 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.6283</v>
+        <v>0.6269</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>-169</v>
+        <v>-168</v>
       </c>
       <c r="H97" s="15" t="n">
-        <v>-188</v>
+        <v>-185</v>
       </c>
       <c r="I97" s="13">
         <f>IF($H$97="","",IF($H$97&lt;0,-$H$97/(-$H$97+100),100/($H$97+100)))</f>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 62.8% (fair -169). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16753,10 +16753,10 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.3717</v>
+        <v>0.3731</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H98" s="15" t="n">
         <v>155</v>
@@ -16783,7 +16783,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 37.2% (fair +169). Your call.</t>
+          <t>Model 37.3% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16951,10 +16951,10 @@
         </is>
       </c>
       <c r="F101" s="13" t="n">
-        <v>0.4492</v>
+        <v>0.4443</v>
       </c>
       <c r="G101" s="14" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H101" s="15" t="n">
         <v>117</v>
@@ -16981,7 +16981,7 @@
       </c>
       <c r="N101" s="19" t="inlineStr">
         <is>
-          <t>Model 44.9% (fair +123). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O101" s="15" t="n"/>
@@ -17017,13 +17017,13 @@
         </is>
       </c>
       <c r="F102" s="13" t="n">
-        <v>0.5508</v>
+        <v>0.5557</v>
       </c>
       <c r="G102" s="14" t="n">
-        <v>-123</v>
+        <v>-125</v>
       </c>
       <c r="H102" s="15" t="n">
-        <v>-117</v>
+        <v>-122</v>
       </c>
       <c r="I102" s="13">
         <f>IF($H$102="","",IF($H$102&lt;0,-$H$102/(-$H$102+100),100/($H$102+100)))</f>
@@ -17047,7 +17047,7 @@
       </c>
       <c r="N102" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O102" s="15" t="n"/>
@@ -17083,10 +17083,10 @@
         </is>
       </c>
       <c r="F103" s="13" t="n">
-        <v>0.51</v>
+        <v>0.5208</v>
       </c>
       <c r="G103" s="14" t="n">
-        <v>-104</v>
+        <v>-109</v>
       </c>
       <c r="H103" s="15" t="n">
         <v>-115</v>
@@ -17113,7 +17113,7 @@
       </c>
       <c r="N103" s="19" t="inlineStr">
         <is>
-          <t>Model 51.0% (fair -104). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O103" s="15" t="n"/>
@@ -17149,10 +17149,10 @@
         </is>
       </c>
       <c r="F104" s="13" t="n">
-        <v>0.49</v>
+        <v>0.4792</v>
       </c>
       <c r="G104" s="14" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H104" s="15" t="n">
         <v>108</v>
@@ -17179,7 +17179,7 @@
       </c>
       <c r="N104" s="19" t="inlineStr">
         <is>
-          <t>Model 49.0% (fair +104). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O104" s="15" t="n"/>
@@ -17215,10 +17215,10 @@
         </is>
       </c>
       <c r="F105" s="13" t="n">
-        <v>0.3755</v>
+        <v>0.3779</v>
       </c>
       <c r="G105" s="14" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H105" s="15" t="n">
         <v>162</v>
@@ -17245,7 +17245,7 @@
       </c>
       <c r="N105" s="19" t="inlineStr">
         <is>
-          <t>Model 37.5% (fair +166). Your call.</t>
+          <t>Model 37.8% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O105" s="15" t="n"/>
@@ -17281,10 +17281,10 @@
         </is>
       </c>
       <c r="F106" s="13" t="n">
-        <v>0.6245000000000001</v>
+        <v>0.6221</v>
       </c>
       <c r="G106" s="14" t="n">
-        <v>-166</v>
+        <v>-165</v>
       </c>
       <c r="H106" s="15" t="n">
         <v>-170</v>
@@ -17311,7 +17311,7 @@
       </c>
       <c r="N106" s="19" t="inlineStr">
         <is>
-          <t>Model 62.5% (fair -166). Your call.</t>
+          <t>Model 62.2% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O106" s="15" t="n"/>
@@ -17347,10 +17347,10 @@
         </is>
       </c>
       <c r="F107" s="13" t="n">
-        <v>0.4256172</v>
+        <v>0.4238366</v>
       </c>
       <c r="G107" s="14" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H107" s="15" t="n">
         <v>138</v>
@@ -17377,7 +17377,7 @@
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>Model 42.6% (fair +135). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O107" s="15" t="n"/>
@@ -17413,10 +17413,10 @@
         </is>
       </c>
       <c r="F108" s="13" t="n">
-        <v>0.5743828</v>
+        <v>0.5761634</v>
       </c>
       <c r="G108" s="14" t="n">
-        <v>-135</v>
+        <v>-136</v>
       </c>
       <c r="H108" s="15" t="n">
         <v>117</v>
@@ -17443,7 +17443,7 @@
       </c>
       <c r="N108" s="19" t="inlineStr">
         <is>
-          <t>Model 57.4% (fair -135). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O108" s="15" t="n"/>
@@ -17479,10 +17479,10 @@
         </is>
       </c>
       <c r="F109" s="13" t="n">
-        <v>0.5676</v>
+        <v>0.5699</v>
       </c>
       <c r="G109" s="14" t="n">
-        <v>-131</v>
+        <v>-133</v>
       </c>
       <c r="H109" s="15" t="n">
         <v>-115</v>
@@ -17509,7 +17509,7 @@
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>Model 56.8% (fair -131). Your call.</t>
+          <t>Model 57.0% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O109" s="15" t="n"/>
@@ -17545,10 +17545,10 @@
         </is>
       </c>
       <c r="F110" s="13" t="n">
-        <v>0.4324</v>
+        <v>0.4301</v>
       </c>
       <c r="G110" s="14" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H110" s="15" t="n">
         <v>108</v>
@@ -17575,7 +17575,7 @@
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>Model 43.2% (fair +131). Your call.</t>
+          <t>Model 43.0% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O110" s="15" t="n"/>
@@ -17611,10 +17611,10 @@
         </is>
       </c>
       <c r="F111" s="13" t="n">
-        <v>0.6472</v>
+        <v>0.6441</v>
       </c>
       <c r="G111" s="14" t="n">
-        <v>-183</v>
+        <v>-181</v>
       </c>
       <c r="H111" s="15" t="n">
         <v>-170</v>
@@ -17641,7 +17641,7 @@
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>Model 64.7% (fair -183). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O111" s="15" t="n"/>
@@ -17677,10 +17677,10 @@
         </is>
       </c>
       <c r="F112" s="13" t="n">
-        <v>0.3528</v>
+        <v>0.3559</v>
       </c>
       <c r="G112" s="14" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H112" s="15" t="n"/>
       <c r="I112" s="13">
@@ -17705,7 +17705,7 @@
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>Model 35.3% (fair +183). Your call.</t>
+          <t>Model 35.6% (fair +181). Your call.</t>
         </is>
       </c>
       <c r="O112" s="15" t="n"/>
@@ -18201,7 +18201,7 @@
         <v>-126</v>
       </c>
       <c r="H120" s="15" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="I120" s="13">
         <f>IF($H$120="","",IF($H$120&lt;0,-$H$120/(-$H$120+100),100/($H$120+100)))</f>
@@ -18521,10 +18521,10 @@
         </is>
       </c>
       <c r="F125" s="13" t="n">
-        <v>0.3488</v>
+        <v>0.3601</v>
       </c>
       <c r="G125" s="14" t="n">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="H125" s="15" t="n"/>
       <c r="I125" s="13">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="N125" s="19" t="inlineStr">
         <is>
-          <t>Model 34.9% (fair +187). Your call.</t>
+          <t>Model 36.0% (fair +178). Your call.</t>
         </is>
       </c>
       <c r="O125" s="15" t="n"/>
@@ -18585,10 +18585,10 @@
         </is>
       </c>
       <c r="F126" s="13" t="n">
-        <v>0.6512</v>
+        <v>0.6399</v>
       </c>
       <c r="G126" s="14" t="n">
-        <v>-187</v>
+        <v>-178</v>
       </c>
       <c r="H126" s="15" t="n"/>
       <c r="I126" s="13">
@@ -18613,7 +18613,7 @@
       </c>
       <c r="N126" s="19" t="inlineStr">
         <is>
-          <t>Model 65.1% (fair -187). Your call.</t>
+          <t>Model 64.0% (fair -178). Your call.</t>
         </is>
       </c>
       <c r="O126" s="15" t="n"/>
@@ -18649,10 +18649,10 @@
         </is>
       </c>
       <c r="F127" s="13" t="n">
-        <v>0.4611</v>
+        <v>0.4688</v>
       </c>
       <c r="G127" s="14" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H127" s="15" t="n"/>
       <c r="I127" s="13">
@@ -18677,7 +18677,7 @@
       </c>
       <c r="N127" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 46.9% (fair +113). Your call.</t>
         </is>
       </c>
       <c r="O127" s="15" t="n"/>
@@ -18713,10 +18713,10 @@
         </is>
       </c>
       <c r="F128" s="13" t="n">
-        <v>0.5389</v>
+        <v>0.5312</v>
       </c>
       <c r="G128" s="14" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="H128" s="15" t="n"/>
       <c r="I128" s="13">
@@ -18741,7 +18741,7 @@
       </c>
       <c r="N128" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 53.1% (fair -113). Your call.</t>
         </is>
       </c>
       <c r="O128" s="15" t="n"/>
@@ -18918,13 +18918,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.2114</v>
+        <v>0.2065</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>373</v>
+        <v>384</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>456</v>
+        <v>495</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -18948,7 +18948,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 21.1% (fair +373). Your call.</t>
+          <t>Model 20.7% (fair +384). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -18984,10 +18984,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.7886</v>
+        <v>0.7935</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-373</v>
+        <v>-384</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-456</v>
@@ -19014,7 +19014,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 78.9% (fair -373). Your call.</t>
+          <t>Model 79.3% (fair -384). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -19050,13 +19050,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.537</v>
+        <v>0.5395</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>100</v>
+        <v>-102</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -19080,7 +19080,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -19116,13 +19116,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.463</v>
+        <v>0.4605</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-102</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -19146,7 +19146,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -19314,13 +19314,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5639000000000001</v>
+        <v>0.5663</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-129</v>
+        <v>-131</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -19344,7 +19344,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -129). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -19380,10 +19380,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4361</v>
+        <v>0.4337</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>-104</v>
@@ -19410,7 +19410,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 43.6% (fair +129). Your call.</t>
+          <t>Model 43.4% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -19446,10 +19446,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.582</v>
+        <v>0.5770999999999999</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-139</v>
+        <v>-136</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>104</v>
@@ -19476,7 +19476,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -19512,13 +19512,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.418</v>
+        <v>0.4229000000000001</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -19542,7 +19542,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -19578,13 +19578,13 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4402</v>
+        <v>0.4396</v>
       </c>
       <c r="G15" s="14" t="n">
         <v>127</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -19644,7 +19644,7 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5598000000000001</v>
+        <v>0.5604</v>
       </c>
       <c r="G16" s="14" t="n">
         <v>-127</v>
@@ -19710,10 +19710,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.7545999999999999</v>
+        <v>0.7556</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-307</v>
+        <v>-309</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>-335</v>
@@ -19740,7 +19740,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 75.5% (fair -307). Your call.</t>
+          <t>Model 75.6% (fair -309). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -19776,13 +19776,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.2454</v>
+        <v>0.2444</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -19806,7 +19806,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 24.5% (fair +307). Your call.</t>
+          <t>Model 24.4% (fair +309). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -19838,17 +19838,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 175.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5797197054418918</v>
+        <v>0.5476</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-138</v>
+        <v>-121</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -19872,7 +19872,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -19904,17 +19904,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 175.5</t>
+          <t>Under 174.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.4202802945581082</v>
+        <v>0.4524</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -19938,7 +19938,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -20046,7 +20046,7 @@
         <v>122</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -20106,13 +20106,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.74107</v>
+        <v>0.7494000000000001</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-286</v>
+        <v>-299</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-285</v>
+        <v>-292</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -20136,7 +20136,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 74.1% (fair -286). Your call.</t>
+          <t>Model 74.9% (fair -299). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -20172,13 +20172,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.25893</v>
+        <v>0.2506</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>335</v>
+        <v>320</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 25.9% (fair +286). Your call.</t>
+          <t>Model 25.1% (fair +299). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -20238,13 +20238,13 @@
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.5816</v>
+        <v>0.5767</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>-139</v>
+        <v>-136</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -20268,7 +20268,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -20304,13 +20304,13 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4184</v>
+        <v>0.4233</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -20334,7 +20334,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -20502,10 +20502,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.6981999999999999</v>
+        <v>0.7000999999999999</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-231</v>
+        <v>-233</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>-257</v>
@@ -20532,7 +20532,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 69.8% (fair -231). Your call.</t>
+          <t>Model 70.0% (fair -233). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -20568,13 +20568,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.3018</v>
+        <v>0.2999</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -20598,7 +20598,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 30.2% (fair +231). Your call.</t>
+          <t>Model 30.0% (fair +233). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -20634,13 +20634,13 @@
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.5326</v>
+        <v>0.5349</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-114</v>
+        <v>-115</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -20664,7 +20664,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 53.5% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -20700,10 +20700,10 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4674</v>
+        <v>0.4651</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -20730,7 +20730,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 46.5% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -20766,13 +20766,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5415</v>
+        <v>0.5522</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-118</v>
+        <v>-123</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -20796,7 +20796,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -20832,13 +20832,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4585</v>
+        <v>0.4478</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-110</v>
+        <v>-104</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -20862,7 +20862,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -20898,13 +20898,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4459</v>
+        <v>0.4471000000000001</v>
       </c>
       <c r="G35" s="14" t="n">
         <v>124</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -20928,7 +20928,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 44.6% (fair +124). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -20964,7 +20964,7 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5541</v>
+        <v>0.5528999999999999</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>-124</v>
@@ -20994,7 +20994,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 55.4% (fair -124). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -21026,17 +21026,17 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Over 180.5</t>
+          <t>Over 180</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.5422</v>
+        <v>0.5479000000000001</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>-118</v>
+        <v>-121</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -21060,7 +21060,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 54.2% (fair -118). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -21092,14 +21092,14 @@
       </c>
       <c r="E38" s="20" t="inlineStr">
         <is>
-          <t>Under 180.5</t>
+          <t>Under 180</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4578</v>
+        <v>0.4292</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="H38" s="15" t="n">
         <v>104</v>
@@ -21126,7 +21126,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 45.8% (fair +118). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -21373,22 +21373,22 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>0.2504</v>
+        <v>0.2503</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>0.4191</v>
+        <v>0.4181</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>-35.25</v>
+        <v>-36.25</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>-8.640000000000001</v>
+        <v>-8.859999999999999</v>
       </c>
       <c r="H5" s="24" t="n">
         <v>5.36</v>
@@ -21404,22 +21404,22 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>0.2502</v>
+        <v>0.2501</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.4231</v>
+        <v>0.4219</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>-31.77</v>
+        <v>-32.77</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>-8.73</v>
+        <v>-8.98</v>
       </c>
       <c r="H6" s="24" t="n">
         <v>7.01</v>
@@ -21508,7 +21508,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>When the model said X%, how often it actually happened (n=356, ECE 0.056 — lower is better; a calibrated model's bars sit on the diagonal).</t>
+          <t>When the model said X%, how often it actually happened (n=357, ECE 0.057 — lower is better; a calibrated model's bars sit on the diagonal).</t>
         </is>
       </c>
     </row>
@@ -21622,16 +21622,16 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>0.543</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.5486</v>
+        <v>0.5517</v>
       </c>
       <c r="E21" s="26" t="n">
-        <v>0.0056</v>
+        <v>0.008800000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -22771,7 +22771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q83"/>
+  <dimension ref="A1:Q82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22788,171 +22788,250 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr">
+        <is>
+          <t>Kansas City Royals offense vs New York Mets defense</t>
+        </is>
+      </c>
+    </row>
     <row r="69">
-      <c r="A69" s="29" t="inlineStr">
-        <is>
-          <t>Kansas City Royals offense vs New York Mets defense</t>
+      <c r="A69" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B69" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D69" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E69" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F69" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G69" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H69" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I69" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J69" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K69" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L69" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M69" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N69" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O69" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P69" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q69" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B70" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C70" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D70" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E70" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F70" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G70" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H70" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I70" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J70" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K70" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L70" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M70" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N70" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O70" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P70" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q70" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="n">
+        <v>4.349</v>
+      </c>
+      <c r="C70" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D70" s="32" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="E70" s="32" t="n">
+        <v>4.733</v>
+      </c>
+      <c r="F70" s="32" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G70" s="32" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H70" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J70" s="36" t="inlineStr">
+        <is>
+          <t>30th</t>
+        </is>
+      </c>
+      <c r="K70" s="32" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="L70" s="32" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="M70" s="32" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="N70" s="32" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="O70" s="32" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="P70" s="32" t="n">
+        <v>4.871</v>
+      </c>
+      <c r="Q70" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B71" s="32" t="n">
-        <v>4.349</v>
-      </c>
-      <c r="C71" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="D71" s="32" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="E71" s="32" t="n">
-        <v>4.733</v>
-      </c>
-      <c r="F71" s="32" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="G71" s="32" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="H71" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I71" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J71" s="36" t="inlineStr">
-        <is>
-          <t>30th</t>
-        </is>
-      </c>
-      <c r="K71" s="32" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="L71" s="32" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="M71" s="32" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="N71" s="32" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="O71" s="32" t="n">
-        <v>6.1</v>
+        <v>7.792</v>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H71" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr"/>
+      <c r="J71" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O71" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P71" s="32" t="n">
-        <v>4.871</v>
+        <v>7.918</v>
       </c>
       <c r="Q71" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B72" s="32" t="n">
-        <v>7.792</v>
+        <v>0.896</v>
       </c>
       <c r="C72" s="32" t="inlineStr">
         <is>
@@ -23016,22 +23095,22 @@
         </is>
       </c>
       <c r="P72" s="32" t="n">
-        <v>7.918</v>
+        <v>0.918</v>
       </c>
       <c r="Q72" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B73" s="32" t="n">
-        <v>0.896</v>
+        <v>8.021000000000001</v>
       </c>
       <c r="C73" s="32" t="inlineStr">
         <is>
@@ -23095,321 +23174,321 @@
         </is>
       </c>
       <c r="P73" s="32" t="n">
-        <v>0.918</v>
+        <v>9.061</v>
       </c>
       <c r="Q73" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B74" s="32" t="n">
-        <v>8.021000000000001</v>
-      </c>
-      <c r="C74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H74" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I74" s="32" t="inlineStr"/>
-      <c r="J74" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O74" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.537</v>
+      </c>
+      <c r="C74" s="32" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="D74" s="32" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E74" s="32" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="F74" s="32" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G74" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H74" s="33" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J74" s="34" t="inlineStr">
+        <is>
+          <t>16th</t>
+        </is>
+      </c>
+      <c r="K74" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L74" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M74" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N74" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O74" s="32" t="n">
+        <v>0.7</v>
       </c>
       <c r="P74" s="32" t="n">
-        <v>9.061</v>
+        <v>0.519</v>
       </c>
       <c r="Q74" s="35" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B75" s="32" t="n">
-        <v>0.537</v>
-      </c>
-      <c r="C75" s="32" t="n">
-        <v>0.867</v>
-      </c>
-      <c r="D75" s="32" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="E75" s="32" t="n">
-        <v>0.867</v>
-      </c>
-      <c r="F75" s="32" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G75" s="32" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H75" s="33" t="inlineStr">
-        <is>
-          <t>1st</t>
-        </is>
-      </c>
-      <c r="I75" s="32" t="inlineStr">
+          <t>Opp 1st Inn R/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>New York Mets offense vs Kansas City Royals defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B77" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D77" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E77" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F77" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H77" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I77" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J77" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K77" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L77" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M77" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N77" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O77" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P77" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q77" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B78" s="32" t="n">
+        <v>4.059</v>
+      </c>
+      <c r="C78" s="32" t="n">
+        <v>4.367</v>
+      </c>
+      <c r="D78" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E78" s="32" t="n">
+        <v>4.667</v>
+      </c>
+      <c r="F78" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="G78" s="32" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H78" s="33" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="J75" s="34" t="inlineStr">
-        <is>
-          <t>16th</t>
-        </is>
-      </c>
-      <c r="K75" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="L75" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M75" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="N75" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O75" s="32" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="P75" s="32" t="n">
-        <v>0.519</v>
-      </c>
-      <c r="Q75" s="35" t="inlineStr">
-        <is>
-          <t>Opp 1st Inn R/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="29" t="inlineStr">
-        <is>
-          <t>New York Mets offense vs Kansas City Royals defense</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B78" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C78" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E78" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F78" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G78" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H78" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I78" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J78" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K78" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L78" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M78" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N78" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O78" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P78" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q78" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="J78" s="34" t="inlineStr">
+        <is>
+          <t>17th</t>
+        </is>
+      </c>
+      <c r="K78" s="32" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="L78" s="32" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="M78" s="32" t="n">
+        <v>6.533</v>
+      </c>
+      <c r="N78" s="32" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="O78" s="32" t="n">
+        <v>5.967</v>
+      </c>
+      <c r="P78" s="32" t="n">
+        <v>5.265</v>
+      </c>
+      <c r="Q78" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Hits/G</t>
         </is>
       </c>
       <c r="B79" s="32" t="n">
-        <v>4.059</v>
-      </c>
-      <c r="C79" s="32" t="n">
-        <v>4.367</v>
-      </c>
-      <c r="D79" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="E79" s="32" t="n">
-        <v>4.667</v>
-      </c>
-      <c r="F79" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="G79" s="32" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="H79" s="33" t="inlineStr">
-        <is>
-          <t>2nd</t>
-        </is>
-      </c>
-      <c r="I79" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J79" s="34" t="inlineStr">
-        <is>
-          <t>17th</t>
-        </is>
-      </c>
-      <c r="K79" s="32" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="L79" s="32" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="M79" s="32" t="n">
-        <v>6.533</v>
-      </c>
-      <c r="N79" s="32" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="O79" s="32" t="n">
-        <v>5.967</v>
+        <v>7.306</v>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="inlineStr"/>
+      <c r="J79" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O79" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="P79" s="32" t="n">
-        <v>5.265</v>
+        <v>8.603999999999999</v>
       </c>
       <c r="Q79" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B80" s="32" t="n">
-        <v>7.306</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
@@ -23473,22 +23552,22 @@
         </is>
       </c>
       <c r="P80" s="32" t="n">
-        <v>8.603999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="Q80" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B81" s="32" t="n">
-        <v>0.9389999999999999</v>
+        <v>8.407999999999999</v>
       </c>
       <c r="C81" s="32" t="inlineStr">
         <is>
@@ -23552,151 +23631,72 @@
         </is>
       </c>
       <c r="P81" s="32" t="n">
-        <v>1.25</v>
+        <v>8.208</v>
       </c>
       <c r="Q81" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B82" s="32" t="n">
-        <v>8.407999999999999</v>
-      </c>
-      <c r="C82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H82" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="inlineStr"/>
-      <c r="J82" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O82" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.556</v>
+      </c>
+      <c r="C82" s="32" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="D82" s="32" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E82" s="32" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="F82" s="32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G82" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" s="33" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J82" s="36" t="inlineStr">
+        <is>
+          <t>24th</t>
+        </is>
+      </c>
+      <c r="K82" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L82" s="32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M82" s="32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N82" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="O82" s="32" t="n">
+        <v>1</v>
       </c>
       <c r="P82" s="32" t="n">
-        <v>8.208</v>
+        <v>0.838</v>
       </c>
       <c r="Q82" s="35" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B83" s="32" t="n">
-        <v>0.556</v>
-      </c>
-      <c r="C83" s="32" t="n">
-        <v>0.5669999999999999</v>
-      </c>
-      <c r="D83" s="32" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E83" s="32" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="F83" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G83" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="H83" s="33" t="inlineStr">
-        <is>
-          <t>6th</t>
-        </is>
-      </c>
-      <c r="I83" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J83" s="36" t="inlineStr">
-        <is>
-          <t>24th</t>
-        </is>
-      </c>
-      <c r="K83" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="L83" s="32" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="M83" s="32" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="N83" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="O83" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="P83" s="32" t="n">
-        <v>0.838</v>
-      </c>
-      <c r="Q83" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>

</xml_diff>